<commit_message>
Add Identity system with User and Role entities
Introduced Role and User entities with EF Core configurations, seeding, and AutoMapper profiles. Updated AgricultureDbContext, seeding logic, and Player to link with User. Refactored Program.cs and reorganized project structure.
</commit_message>
<xml_diff>
--- a/src/External/Agriculture.Seeding/Data/GardenData.xlsx
+++ b/src/External/Agriculture.Seeding/Data/GardenData.xlsx
@@ -5,13 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Farms" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="FarmPlots" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="PlayerFarms" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Roles" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Users" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="27">
   <si>
     <t xml:space="preserve">UserName</t>
   </si>
@@ -71,6 +73,39 @@
   </si>
   <si>
     <t xml:space="preserve">IsActive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperAdmin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has full access to the game system, including system configuration, player management, and game data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages players, farms, game content, and general game operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moderator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitors player activities and handles reports, inappropriate content, and player-related issues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Player</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A player who owns and manages farms, grows crops, collects resources, and participates in game activities.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PasswordHash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RoleName</t>
   </si>
 </sst>
 </file>
@@ -103,9 +138,11 @@
       <family val="0"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -150,7 +187,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -159,7 +196,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -331,8 +376,8 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="14.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="15.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -348,7 +393,7 @@
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -365,7 +410,7 @@
       <c r="D2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -584,4 +629,116 @@
     <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="89.71"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.7"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>123456</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>